<commit_message>
feat: pipeline consolidation - ubj and surgery insurance
</commit_message>
<xml_diff>
--- a/insurance_data/2_care/home_facility/extracted_data.xlsx
+++ b/insurance_data/2_care/home_facility/extracted_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT43"/>
+  <dimension ref="A1:AT53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6736,6 +6736,2126 @@
       <c r="AS43" t="inlineStr"/>
       <c r="AT43" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>주계약</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>사망 보험금</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1000만원  원</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1000만원  원</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>28,300 원</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>24,700 원</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>주계약</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>사망 보험금</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>피보험자가 보험기간 중 사망하였을 경우</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>1000만원[단, 피보험자가 계약일부터 1년 이내에 재해 이외의 원인으로 사망하였을 경우에는 보험가입금액의 50%]</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>1000만원  원</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>28300  원</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>24,700  원</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>2.25 %</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>106.3 %</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>106.8 %</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI44" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO44" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP44" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ44" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR44" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : - 30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)재가급여지원 특약T(무배당,저 해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>9,250 원</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>15,210 원</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)재가급여지원 특약T(무배당,저 해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 「장기요양상태 보장개시일」 이후에 최초로 "장기요양상태(1-5등급)"로 판정 확정되고, 그 날 로부터 이 특약의 보험기간동안 재가급여를 이용하였을 경우 (발 생후 보험월 기준 월1회 한)</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>(1회당) 10만원</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>9250  원</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>15,210  원</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>2.25 %</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>106.3 %</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>106.8 %</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP45" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ45" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR45" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : - 30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT45" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>장기요양(1-인지지원등급)재가급 여지원특약T(무배당,저해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>9,880 원</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>16,000 원</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>장기요양(1-인지지원등급)재가급 여지원특약T(무배당,저해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 「장기요양상태 보장개시일」 이후에 최초로 "장기요양상태(1-인지지원등급)"로 판정 확정되고, 그 날로부터 이 특약의 보험기간동안 재가급여를 이용하였을 경우 (발생후 보험월 기준 월1회 한)</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>(1회당) 10만원</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>9880  원</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>16,000  원</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>2.25 %</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>106.3 %</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>106.8 %</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI46" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO46" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP46" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ46" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR46" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : - 30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT46" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)시설급여지원 특약T(무배당,저해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2,560 원</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>5,530 원</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)시설급여지원 특약T(무배당,저해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 「장기요양상태 보장개시일」 이후에 최초로 "장기요양상태(1-5등급)"로 판정 확정되고, 그 날 로부터 이 특약의 보험기간동안 시설급여를 이용하였을 경우 (발 생후 보험월 기준 월1회 한)</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>(1회당) 10만원</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>2560  원</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>5,530  원</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>2.25 %</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>106.3 %</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>106.8 %</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI47" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO47" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP47" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ47" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR47" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : - 30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT47" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>입원간병인사용 (180일한도,요양 병원제외)특약 T(무배당,저해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2,540 원</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>3,310 원</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>삼성 간편 웰에이징(Well-Aging) 건강보험 (2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>입원간병인사용 (180일한도,요양 병원제외)특약 T(무배당,저해약환급금형)[간편고지형]</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 질병 또는 재해로 인하여 그 직접적인 치료를 목적으로 1일 이상 계속하여 병원(단, 요양병원 제외)에 입원하며 간병인을 사용하였을 경우 (1회 입원당 사용일수는 180일한도) ※ 단, 재해 이외의 원인으로 인한 입원시 1년 이내 50% 삭감 지급함</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>간병인 사용금액이 1일당 7万 미만인 경우 (1일당) 5만원 / 간병인 사용금액이 1일당 7万 이상인 경우 (1일당)10만원</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>2540  원</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>3,310  원</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>2.25 %</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>106.3 %</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>106.8 %</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO48" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP48" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ48" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR48" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS48" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : - 30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT48" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>주계약</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>사망보험금</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1000만원  원</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>1000만원  원</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>24,400 원</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>21,900 원</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>주계약</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>사망보험금</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>사망시</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>1000만원</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>1000만원  원</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>24400  원</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>21,900  원</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>2.15 %</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>110.0 %</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>110.5 %</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI49" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO49" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP49" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ49" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR49" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : -30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 100만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT49" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)재가급여지원특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>8,730 원</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>13,360 원</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)재가급여지원특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>-피보험자가 이 특약의 보험기간 중 「장기요양상태 보장개시일」 이후에 최초로 "장기요양상태(1-5등급)"로 판정 확정되고, 그 날 로부터 이 특약의 보험기간동안 재가급여를 이용하였을 경우 (발 생후 보험월 기준 월1회 한)</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>(1회당) 10만원</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>8730  원</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>13,360  원</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>2.15 %</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>110.0 %</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>110.5 %</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO50" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP50" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ50" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR50" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : -30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 100만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT50" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>장기요양(1-인지지원등급)재가급여지원특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>9,290 원</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>14,100 원</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>장기요양(1-인지지원등급)재가급여지원특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 「장기요양상태 보장개시일」 이후에 최초로 "장기요양상태(1-인지지원등급)"로 판정 확정되고, 그 날로부터 이 특약의 보험기간동안 재가급여를 이용하였을 경우 (발생후 보험월 기준 월1회 한)</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>(1회당) 10만원</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>9290  원</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>14,100  원</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>2.15 %</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>110.0 %</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>110.5 %</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI51" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO51" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP51" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ51" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR51" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : -30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 100만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)시설급여지원특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2,470 원</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>5,210 원</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>장기요양(1-5등급)시설급여지원특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 「장기요양상태 보장개시일」 이후에 최초로 "장기요양상태(1-5등급)"로 판정 확정되고, 그 날 로부터 이 특약의 보험기간동안 시설급여를 이용하였을 경우 (발 생후 보험월 기준 월1회 한)</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>(1회당) 10만원</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>10만원  원</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>2470  원</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>5,210  원</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>2.15 %</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>110.0 %</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>110.5 %</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO52" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP52" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR52" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : -30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 100만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>입원간병인사용 (180일한도,요양병원)특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1만원  원</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>1만원  원</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2,060 원</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>3,260 원</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>보장성_상품비교_20260608162031320.xls</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>삼성웰에이징(Well-Aging)건강보험(2601)(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>특약</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>입원간병인사용 (180일한도,요양병원)특약P(무배당,저해약환급금형)</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>피보험자가 이 특약의 보험기간 중 질병 또는 재해로 인하여 그 직접적인 치료를 목적으로 1일 이상 계속하여 요양병원에 입원하 며 간병인을 사용하였을 경우 (1회 입원당 사용일수는 180일한도)</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>(1일당)1만원</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>1만원  원</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>2060  원</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>3,260  원</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>2.15 %</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>110.0 %</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>110.5 %</t>
+        </is>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI53" t="inlineStr">
+        <is>
+          <t>기본형</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>무해지/저해지환급</t>
+        </is>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AO53" t="inlineStr">
+        <is>
+          <t>비갱신형</t>
+        </is>
+      </c>
+      <c r="AP53" t="inlineStr">
+        <is>
+          <t>비유니버셜</t>
+        </is>
+      </c>
+      <c r="AQ53" t="inlineStr">
+        <is>
+          <t>대면채널</t>
+        </is>
+      </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>□ 필수기재사항 1. 가입나이 : -30세 ~ 최대 75세 ※ 납입기간별로 가입나이는 차이가 있을 수 있습니다. 2. 보험기간 : 종신 3. 보험료 예시기준 - 주보험 보험가입금액 1,000만원, 40세, 종신, 20년납, 월납, 2종(일반고지형) □ 선택기재사항 1. 보험료 납입기간 :  - 10,15,20,30년납 2. 보험가격지수 예시기준 :  - 주보험 보험가입금액 100만원, 40세, 종신, 20년납, 월납, 2종(일반고지형)  ※ 보다 자세한 내용은 상품요약서 및 기초서류 참고</t>
+        </is>
+      </c>
+      <c r="AT53" t="inlineStr">
+        <is>
+          <t>1588-3114</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>